<commit_message>
modal & orders loader
</commit_message>
<xml_diff>
--- a/public/templates/kp-template-1.xlsx
+++ b/public/templates/kp-template-1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mp-calc-2.0\price-calc\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1226F845-1AD9-4FE7-A1D8-F5EC50F01719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE217EC5-7CA0-46FD-9707-F44F5137FDF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5790" yWindow="5790" windowWidth="23160" windowHeight="11910" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="КП-1 (с НДС) RUS" sheetId="16" r:id="rId1"/>
@@ -807,6 +807,48 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
@@ -816,30 +858,6 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -864,32 +882,14 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1302,57 +1302,57 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="60" t="s">
+      <c r="C1" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
     </row>
     <row r="2" spans="1:6" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="60"/>
-      <c r="D4" s="60"/>
-      <c r="E4" s="60"/>
-      <c r="F4" s="60"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C5" s="60"/>
-      <c r="D5" s="60"/>
-      <c r="E5" s="60"/>
-      <c r="F5" s="60"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="60"/>
-      <c r="D6" s="60"/>
-      <c r="E6" s="60"/>
-      <c r="F6" s="60"/>
+      <c r="C6" s="36"/>
+      <c r="D6" s="36"/>
+      <c r="E6" s="36"/>
+      <c r="F6" s="36"/>
     </row>
     <row r="7" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="60"/>
-      <c r="D7" s="60"/>
-      <c r="E7" s="60"/>
-      <c r="F7" s="60"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="60"/>
-      <c r="D8" s="60"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="60"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
@@ -1363,40 +1363,40 @@
       <c r="F9" s="9"/>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="34" t="s">
+      <c r="A10" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="34"/>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
+      <c r="B10" s="48"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
     </row>
     <row r="11" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="33"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="33"/>
-      <c r="F11" s="33"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="47"/>
     </row>
     <row r="12" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="35"/>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="35"/>
+      <c r="A12" s="49"/>
+      <c r="B12" s="49"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="49"/>
+      <c r="F12" s="49"/>
     </row>
     <row r="13" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="35"/>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
+      <c r="A13" s="49"/>
+      <c r="B13" s="49"/>
+      <c r="C13" s="49"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="49"/>
+      <c r="F13" s="49"/>
     </row>
     <row r="14" spans="1:6" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
@@ -1409,30 +1409,30 @@
       <c r="F14" s="4"/>
     </row>
     <row r="15" spans="1:6" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="53" t="s">
+      <c r="A15" s="44" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="53"/>
-      <c r="C15" s="53"/>
-      <c r="D15" s="53"/>
-      <c r="E15" s="53"/>
-      <c r="F15" s="53"/>
+      <c r="B15" s="44"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
     </row>
     <row r="16" spans="1:6" s="13" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="53"/>
-      <c r="B16" s="53"/>
-      <c r="C16" s="53"/>
-      <c r="D16" s="53"/>
-      <c r="E16" s="53"/>
-      <c r="F16" s="53"/>
+      <c r="A16" s="44"/>
+      <c r="B16" s="44"/>
+      <c r="C16" s="44"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="44"/>
     </row>
     <row r="17" spans="1:6" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="53"/>
-      <c r="B17" s="53"/>
-      <c r="C17" s="53"/>
-      <c r="D17" s="53"/>
-      <c r="E17" s="53"/>
-      <c r="F17" s="53"/>
+      <c r="A17" s="44"/>
+      <c r="B17" s="44"/>
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="44"/>
+      <c r="F17" s="44"/>
     </row>
     <row r="18" spans="1:6" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
@@ -1453,30 +1453,30 @@
       <c r="F19" s="4"/>
     </row>
     <row r="20" spans="1:6" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="54" t="s">
+      <c r="A20" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="54"/>
-      <c r="C20" s="54"/>
-      <c r="D20" s="54"/>
-      <c r="E20" s="54"/>
-      <c r="F20" s="54"/>
+      <c r="B20" s="45"/>
+      <c r="C20" s="45"/>
+      <c r="D20" s="45"/>
+      <c r="E20" s="45"/>
+      <c r="F20" s="45"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="54"/>
-      <c r="B21" s="54"/>
-      <c r="C21" s="54"/>
-      <c r="D21" s="54"/>
-      <c r="E21" s="54"/>
-      <c r="F21" s="54"/>
+      <c r="A21" s="45"/>
+      <c r="B21" s="45"/>
+      <c r="C21" s="45"/>
+      <c r="D21" s="45"/>
+      <c r="E21" s="45"/>
+      <c r="F21" s="45"/>
     </row>
     <row r="22" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="54"/>
-      <c r="B22" s="54"/>
-      <c r="C22" s="54"/>
-      <c r="D22" s="54"/>
-      <c r="E22" s="54"/>
-      <c r="F22" s="54"/>
+      <c r="A22" s="45"/>
+      <c r="B22" s="45"/>
+      <c r="C22" s="45"/>
+      <c r="D22" s="45"/>
+      <c r="E22" s="45"/>
+      <c r="F22" s="45"/>
     </row>
     <row r="23" spans="1:6" s="11" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3"/>
@@ -1547,70 +1547,70 @@
       </c>
     </row>
     <row r="30" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="55" t="s">
+      <c r="A30" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="55"/>
-      <c r="C30" s="55"/>
-      <c r="D30" s="55"/>
-      <c r="E30" s="55"/>
-      <c r="F30" s="55"/>
+      <c r="B30" s="46"/>
+      <c r="C30" s="46"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="46"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="55"/>
-      <c r="B31" s="55"/>
-      <c r="C31" s="55"/>
-      <c r="D31" s="55"/>
-      <c r="E31" s="55"/>
-      <c r="F31" s="55"/>
+      <c r="A31" s="46"/>
+      <c r="B31" s="46"/>
+      <c r="C31" s="46"/>
+      <c r="D31" s="46"/>
+      <c r="E31" s="46"/>
+      <c r="F31" s="46"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="55"/>
-      <c r="B32" s="55"/>
-      <c r="C32" s="55"/>
-      <c r="D32" s="55"/>
-      <c r="E32" s="55"/>
-      <c r="F32" s="55"/>
+      <c r="A32" s="46"/>
+      <c r="B32" s="46"/>
+      <c r="C32" s="46"/>
+      <c r="D32" s="46"/>
+      <c r="E32" s="46"/>
+      <c r="F32" s="46"/>
     </row>
     <row r="33" spans="1:6" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="52" t="s">
+      <c r="A33" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="B33" s="52"/>
-      <c r="C33" s="52"/>
-      <c r="D33" s="52"/>
+      <c r="B33" s="37"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="37"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
     </row>
     <row r="34" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="52"/>
-      <c r="B34" s="52"/>
-      <c r="C34" s="52"/>
-      <c r="D34" s="52"/>
+      <c r="A34" s="37"/>
+      <c r="B34" s="37"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="37"/>
     </row>
     <row r="35" spans="1:6" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="36"/>
-      <c r="B35" s="36"/>
-      <c r="C35" s="36"/>
-      <c r="D35" s="36"/>
-      <c r="E35" s="36"/>
-      <c r="F35" s="36"/>
+      <c r="A35" s="34"/>
+      <c r="B35" s="34"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="34"/>
+      <c r="E35" s="34"/>
+      <c r="F35" s="34"/>
     </row>
     <row r="36" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="36"/>
-      <c r="B36" s="36"/>
-      <c r="C36" s="36"/>
-      <c r="D36" s="36"/>
-      <c r="E36" s="36"/>
-      <c r="F36" s="36"/>
+      <c r="A36" s="34"/>
+      <c r="B36" s="34"/>
+      <c r="C36" s="34"/>
+      <c r="D36" s="34"/>
+      <c r="E36" s="34"/>
+      <c r="F36" s="34"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="36"/>
-      <c r="B37" s="36"/>
-      <c r="C37" s="36"/>
-      <c r="D37" s="36"/>
-      <c r="E37" s="36"/>
-      <c r="F37" s="36"/>
+      <c r="A37" s="34"/>
+      <c r="B37" s="34"/>
+      <c r="C37" s="34"/>
+      <c r="D37" s="34"/>
+      <c r="E37" s="34"/>
+      <c r="F37" s="34"/>
     </row>
     <row r="39" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="4" t="s">
@@ -1628,16 +1628,16 @@
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B42" s="37" t="s">
+      <c r="B42" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="C42" s="37"/>
+      <c r="C42" s="35"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B43" s="37" t="s">
+      <c r="B43" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="C43" s="37"/>
+      <c r="C43" s="35"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45"/>
@@ -2051,15 +2051,15 @@
     <mergeCell ref="A15:F17"/>
     <mergeCell ref="A20:F22"/>
     <mergeCell ref="A30:F32"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A13:F13"/>
     <mergeCell ref="A37:F37"/>
     <mergeCell ref="B42:C42"/>
     <mergeCell ref="B43:C43"/>
     <mergeCell ref="A35:F35"/>
     <mergeCell ref="A36:F36"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A13:F13"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.11811023622047245" footer="0.19685039370078741"/>
@@ -2083,8 +2083,8 @@
     <col min="5" max="5" width="12.28515625" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.28515625" style="3" customWidth="1"/>
     <col min="7" max="7" width="7.140625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" style="3" customWidth="1"/>
-    <col min="9" max="9" width="15.140625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="14.140625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="16.5703125" style="3" customWidth="1"/>
     <col min="10" max="10" width="19.7109375" style="3" customWidth="1"/>
     <col min="11" max="16384" width="9.140625" style="3"/>
   </cols>
@@ -2169,52 +2169,52 @@
       <c r="I9" s="9"/>
     </row>
     <row r="10" spans="1:10" ht="21" x14ac:dyDescent="0.25">
-      <c r="A10" s="34" t="s">
+      <c r="A10" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="34"/>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="34"/>
-      <c r="I10" s="34"/>
+      <c r="B10" s="48"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
+      <c r="G10" s="48"/>
+      <c r="H10" s="48"/>
+      <c r="I10" s="48"/>
     </row>
     <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="33"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="33"/>
-      <c r="F11" s="33"/>
-      <c r="G11" s="33"/>
-      <c r="H11" s="33"/>
-      <c r="I11" s="33"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="47"/>
+      <c r="I11" s="47"/>
     </row>
     <row r="12" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="35"/>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="35"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="35"/>
-      <c r="I12" s="35"/>
+      <c r="A12" s="49"/>
+      <c r="B12" s="49"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="49"/>
+      <c r="F12" s="49"/>
+      <c r="G12" s="49"/>
+      <c r="H12" s="49"/>
+      <c r="I12" s="49"/>
     </row>
     <row r="13" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="35"/>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="35"/>
-      <c r="H13" s="35"/>
-      <c r="I13" s="35"/>
+      <c r="A13" s="49"/>
+      <c r="B13" s="49"/>
+      <c r="C13" s="49"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="49"/>
+      <c r="F13" s="49"/>
+      <c r="G13" s="49"/>
+      <c r="H13" s="49"/>
+      <c r="I13" s="49"/>
     </row>
     <row r="14" spans="1:10" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
@@ -2230,40 +2230,40 @@
       <c r="I14" s="4"/>
     </row>
     <row r="15" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="53" t="s">
+      <c r="A15" s="44" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="53"/>
-      <c r="C15" s="53"/>
-      <c r="D15" s="53"/>
-      <c r="E15" s="53"/>
-      <c r="F15" s="53"/>
-      <c r="G15" s="53"/>
-      <c r="H15" s="53"/>
-      <c r="I15" s="53"/>
+      <c r="B15" s="44"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="44"/>
       <c r="J15" s="14"/>
     </row>
     <row r="16" spans="1:10" s="13" customFormat="1" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="53"/>
-      <c r="B16" s="53"/>
-      <c r="C16" s="53"/>
-      <c r="D16" s="53"/>
-      <c r="E16" s="53"/>
-      <c r="F16" s="53"/>
-      <c r="G16" s="53"/>
-      <c r="H16" s="53"/>
-      <c r="I16" s="53"/>
+      <c r="A16" s="44"/>
+      <c r="B16" s="44"/>
+      <c r="C16" s="44"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="44"/>
+      <c r="G16" s="44"/>
+      <c r="H16" s="44"/>
+      <c r="I16" s="44"/>
     </row>
     <row r="17" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="53"/>
-      <c r="B17" s="53"/>
-      <c r="C17" s="53"/>
-      <c r="D17" s="53"/>
-      <c r="E17" s="53"/>
-      <c r="F17" s="53"/>
-      <c r="G17" s="53"/>
-      <c r="H17" s="53"/>
-      <c r="I17" s="53"/>
+      <c r="A17" s="44"/>
+      <c r="B17" s="44"/>
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="44"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="44"/>
+      <c r="H17" s="44"/>
+      <c r="I17" s="44"/>
     </row>
     <row r="18" spans="1:9" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
@@ -2284,45 +2284,45 @@
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="56"/>
+      <c r="F19" s="33"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
     </row>
     <row r="20" spans="1:9" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="57" t="s">
+      <c r="A20" s="60" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="57"/>
-      <c r="C20" s="57"/>
-      <c r="D20" s="57"/>
-      <c r="E20" s="57"/>
-      <c r="F20" s="57"/>
-      <c r="G20" s="57"/>
-      <c r="H20" s="57"/>
-      <c r="I20" s="57"/>
+      <c r="B20" s="60"/>
+      <c r="C20" s="60"/>
+      <c r="D20" s="60"/>
+      <c r="E20" s="60"/>
+      <c r="F20" s="60"/>
+      <c r="G20" s="60"/>
+      <c r="H20" s="60"/>
+      <c r="I20" s="60"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="57"/>
-      <c r="B21" s="57"/>
-      <c r="C21" s="57"/>
-      <c r="D21" s="57"/>
-      <c r="E21" s="57"/>
-      <c r="F21" s="57"/>
-      <c r="G21" s="57"/>
-      <c r="H21" s="57"/>
-      <c r="I21" s="57"/>
+      <c r="A21" s="60"/>
+      <c r="B21" s="60"/>
+      <c r="C21" s="60"/>
+      <c r="D21" s="60"/>
+      <c r="E21" s="60"/>
+      <c r="F21" s="60"/>
+      <c r="G21" s="60"/>
+      <c r="H21" s="60"/>
+      <c r="I21" s="60"/>
     </row>
     <row r="22" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="57"/>
-      <c r="B22" s="57"/>
-      <c r="C22" s="57"/>
-      <c r="D22" s="57"/>
-      <c r="E22" s="57"/>
-      <c r="F22" s="57"/>
-      <c r="G22" s="57"/>
-      <c r="H22" s="57"/>
-      <c r="I22" s="57"/>
+      <c r="A22" s="60"/>
+      <c r="B22" s="60"/>
+      <c r="C22" s="60"/>
+      <c r="D22" s="60"/>
+      <c r="E22" s="60"/>
+      <c r="F22" s="60"/>
+      <c r="G22" s="60"/>
+      <c r="H22" s="60"/>
+      <c r="I22" s="60"/>
     </row>
     <row r="23" spans="1:9" s="11" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3"/>
@@ -2336,10 +2336,10 @@
       <c r="I23" s="3"/>
     </row>
     <row r="24" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="50" t="s">
+      <c r="A24" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="B24" s="46" t="s">
+      <c r="B24" s="52" t="s">
         <v>2</v>
       </c>
       <c r="C24" s="40" t="s">
@@ -2354,28 +2354,28 @@
       <c r="F24" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="G24" s="44" t="s">
+      <c r="G24" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="H24" s="45"/>
+      <c r="H24" s="51"/>
       <c r="I24" s="40" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:9" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="51"/>
-      <c r="B25" s="46"/>
-      <c r="C25" s="46"/>
-      <c r="D25" s="46"/>
-      <c r="E25" s="46"/>
-      <c r="F25" s="46"/>
+      <c r="A25" s="57"/>
+      <c r="B25" s="52"/>
+      <c r="C25" s="52"/>
+      <c r="D25" s="52"/>
+      <c r="E25" s="52"/>
+      <c r="F25" s="52"/>
       <c r="G25" s="29" t="s">
         <v>22</v>
       </c>
       <c r="H25" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="I25" s="46"/>
+      <c r="I25" s="52"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="30">
@@ -2402,16 +2402,16 @@
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="47" t="s">
+      <c r="A27" s="53" t="s">
         <v>18</v>
       </c>
-      <c r="B27" s="48"/>
-      <c r="C27" s="48"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="48"/>
-      <c r="H27" s="49"/>
+      <c r="B27" s="54"/>
+      <c r="C27" s="54"/>
+      <c r="D27" s="54"/>
+      <c r="E27" s="54"/>
+      <c r="F27" s="54"/>
+      <c r="G27" s="54"/>
+      <c r="H27" s="55"/>
       <c r="I27" s="27">
         <f>SUM(I26:I26)</f>
         <v>0</v>
@@ -2423,92 +2423,92 @@
       </c>
     </row>
     <row r="30" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="53" t="s">
+      <c r="A30" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="53"/>
-      <c r="C30" s="53"/>
-      <c r="D30" s="53"/>
-      <c r="E30" s="53"/>
-      <c r="F30" s="53"/>
-      <c r="G30" s="53"/>
-      <c r="H30" s="53"/>
-      <c r="I30" s="53"/>
+      <c r="B30" s="44"/>
+      <c r="C30" s="44"/>
+      <c r="D30" s="44"/>
+      <c r="E30" s="44"/>
+      <c r="F30" s="44"/>
+      <c r="G30" s="44"/>
+      <c r="H30" s="44"/>
+      <c r="I30" s="44"/>
     </row>
     <row r="31" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="53"/>
-      <c r="B31" s="53"/>
-      <c r="C31" s="53"/>
-      <c r="D31" s="53"/>
-      <c r="E31" s="53"/>
-      <c r="F31" s="53"/>
-      <c r="G31" s="53"/>
-      <c r="H31" s="53"/>
-      <c r="I31" s="53"/>
+      <c r="A31" s="44"/>
+      <c r="B31" s="44"/>
+      <c r="C31" s="44"/>
+      <c r="D31" s="44"/>
+      <c r="E31" s="44"/>
+      <c r="F31" s="44"/>
+      <c r="G31" s="44"/>
+      <c r="H31" s="44"/>
+      <c r="I31" s="44"/>
     </row>
     <row r="32" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="53"/>
-      <c r="B32" s="53"/>
-      <c r="C32" s="53"/>
-      <c r="D32" s="53"/>
-      <c r="E32" s="53"/>
-      <c r="F32" s="53"/>
-      <c r="G32" s="53"/>
-      <c r="H32" s="53"/>
-      <c r="I32" s="53"/>
+      <c r="A32" s="44"/>
+      <c r="B32" s="44"/>
+      <c r="C32" s="44"/>
+      <c r="D32" s="44"/>
+      <c r="E32" s="44"/>
+      <c r="F32" s="44"/>
+      <c r="G32" s="44"/>
+      <c r="H32" s="44"/>
+      <c r="I32" s="44"/>
     </row>
     <row r="33" spans="1:9" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="52" t="s">
+      <c r="A33" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="B33" s="52"/>
-      <c r="C33" s="52"/>
-      <c r="D33" s="52"/>
-      <c r="E33" s="52"/>
+      <c r="B33" s="37"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="37"/>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
     </row>
     <row r="34" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="52"/>
-      <c r="B34" s="52"/>
-      <c r="C34" s="52"/>
-      <c r="D34" s="52"/>
-      <c r="E34" s="52"/>
+      <c r="A34" s="37"/>
+      <c r="B34" s="37"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="37"/>
+      <c r="E34" s="37"/>
     </row>
     <row r="35" spans="1:9" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="36"/>
-      <c r="B35" s="36"/>
-      <c r="C35" s="36"/>
-      <c r="D35" s="36"/>
-      <c r="E35" s="36"/>
-      <c r="F35" s="36"/>
-      <c r="G35" s="36"/>
-      <c r="H35" s="36"/>
-      <c r="I35" s="36"/>
+      <c r="A35" s="34"/>
+      <c r="B35" s="34"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="34"/>
+      <c r="E35" s="34"/>
+      <c r="F35" s="34"/>
+      <c r="G35" s="34"/>
+      <c r="H35" s="34"/>
+      <c r="I35" s="34"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="36"/>
-      <c r="B36" s="36"/>
-      <c r="C36" s="36"/>
-      <c r="D36" s="36"/>
-      <c r="E36" s="36"/>
-      <c r="F36" s="36"/>
-      <c r="G36" s="36"/>
-      <c r="H36" s="36"/>
-      <c r="I36" s="36"/>
+      <c r="A36" s="34"/>
+      <c r="B36" s="34"/>
+      <c r="C36" s="34"/>
+      <c r="D36" s="34"/>
+      <c r="E36" s="34"/>
+      <c r="F36" s="34"/>
+      <c r="G36" s="34"/>
+      <c r="H36" s="34"/>
+      <c r="I36" s="34"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="36"/>
-      <c r="B37" s="36"/>
-      <c r="C37" s="36"/>
-      <c r="D37" s="36"/>
-      <c r="E37" s="36"/>
-      <c r="F37" s="36"/>
-      <c r="G37" s="36"/>
-      <c r="H37" s="36"/>
-      <c r="I37" s="36"/>
+      <c r="A37" s="34"/>
+      <c r="B37" s="34"/>
+      <c r="C37" s="34"/>
+      <c r="D37" s="34"/>
+      <c r="E37" s="34"/>
+      <c r="F37" s="34"/>
+      <c r="G37" s="34"/>
+      <c r="H37" s="34"/>
+      <c r="I37" s="34"/>
     </row>
     <row r="39" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="4" t="s">
@@ -2516,10 +2516,10 @@
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B40" s="37" t="s">
+      <c r="B40" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="C40" s="37"/>
+      <c r="C40" s="35"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B41" s="4" t="s">
@@ -2527,18 +2527,18 @@
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B42" s="37" t="s">
+      <c r="B42" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="C42" s="37"/>
-      <c r="D42" s="37"/>
+      <c r="C42" s="35"/>
+      <c r="D42" s="35"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B43" s="37" t="s">
+      <c r="B43" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="C43" s="37"/>
-      <c r="D43" s="37"/>
+      <c r="C43" s="35"/>
+      <c r="D43" s="35"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I44" s="3" t="s">

</xml_diff>

<commit_message>
kp checks label fix
</commit_message>
<xml_diff>
--- a/public/templates/kp-template-1.xlsx
+++ b/public/templates/kp-template-1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mp-calc-2.0\price-calc\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE217EC5-7CA0-46FD-9707-F44F5137FDF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBA45A5D-B9A0-4B34-9CDE-65DD5BCC8504}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="33">
   <si>
     <t>№</t>
   </si>
@@ -162,6 +162,14 @@
 Тел.: +99871291-37-75.Р/с 2020 8000 3048 2507 1001
 в ОПЕРУ АКБ «ASIA ALLIANCE BANK», МФО 01095
                                        ИНН 301262117 ОКЭД 46730 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">☐ В наличии    ☐ Комплексность    ☐ Временное хранение    ☐ Скидка    ☐ Доставка       
+☐ Шеф. Монтаж    ☐ Эксклюзивность    ☐ Ускоренная поставка    ☐ Доп. скидка    ☐ PMG    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">☐ Фундамент    ☐ Фасад    ☐ СК    ☐ ЛКМ    ☐ Звукоизоляция    ☐ Линейный водоотвод   
+☐ Мансарда    ☐ Терраса    ☐ ПК    ☐ Полы    ☐ Опалубочная система    </t>
   </si>
 </sst>
 </file>
@@ -2231,7 +2239,7 @@
     </row>
     <row r="15" spans="1:10" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="44" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B15" s="44"/>
       <c r="C15" s="44"/>
@@ -2424,7 +2432,7 @@
     </row>
     <row r="30" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="44" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B30" s="44"/>
       <c r="C30" s="44"/>

</xml_diff>